<commit_message>
feat(import): remove unique_id from templates, auto-generate from coordinates, and skip duplicate records with warning
</commit_message>
<xml_diff>
--- a/backend/app/templates/previous_records_template.xlsx
+++ b/backend/app/templates/previous_records_template.xlsx
@@ -449,33 +449,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="51" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
-    <col width="31" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="25" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="30" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="34" customWidth="1" min="22" max="22"/>
-    <col width="36" customWidth="1" min="23" max="23"/>
-    <col width="53" customWidth="1" min="24" max="24"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="36" customWidth="1" min="21" max="21"/>
+    <col width="53" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -486,115 +484,105 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>visit_order</t>
+          <t>coordinates</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>unique_id</t>
+          <t>site_address</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>coordinates</t>
+          <t>street_address</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>site_address</t>
+          <t>village</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>street_address</t>
+          <t>taluk</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>village</t>
+          <t>district</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>taluk</t>
+          <t>survey_no</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>subdivision_no</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>survey_no</t>
+          <t>land_use</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>subdivision_no</t>
+          <t>owner_name_en</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>land_use</t>
+          <t>date_of_visit</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>owner_name_en</t>
+          <t>construction_happening</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>cumulative_road_distance_km</t>
+          <t>type_of_construction</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>date_of_visit</t>
+          <t>stage_of_construction</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>construction_happening</t>
+          <t>building_user_name</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>type_of_construction</t>
+          <t>relationship_with_building</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>stage_of_construction</t>
+          <t>spoken_with</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>building_user_name</t>
+          <t>contact_number</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>relationship_with_building</t>
+          <t>site_contractor_architect_name</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>contact_number</t>
+          <t>site_contractor_architect_number</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>site_contractor_architect_name</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>site_contractor_architect_number</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
@@ -606,115 +594,107 @@
           <t>operator1@company.com</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>1</v>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>11.016844, 76.955832</t>
+        </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>PREV-1001</t>
+          <t>142/3A, Trichy Road, Kurichy, Coimbatore</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>11.016844, 76.955832</t>
+          <t>Trichy Road</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>142/3A, Trichy Road, Kurichy, Coimbatore</t>
+          <t>Kurichy</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Trichy Road</t>
+          <t>Coimbatore South</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kurichy</t>
+          <t>Coimbatore</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Coimbatore South</t>
+          <t>142/3A</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>142/3A</t>
+          <t>Residential</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Ramesh Kumar</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
+          <t>2024-03-15</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
           <t>Residential</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Roof Level</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Ramesh Kumar</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>2024-03-15</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Residential</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Roof Level</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>Ramesh Kumar</t>
+          <t>9876543210</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Suresh Builders</t>
         </is>
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>9876500001</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
-        <is>
-          <t>Suresh Builders</t>
-        </is>
-      </c>
-      <c r="W2" s="2" t="inlineStr">
-        <is>
-          <t>9876500001</t>
-        </is>
-      </c>
-      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>Construction in progress, boundary wall completed</t>
         </is>
@@ -726,107 +706,99 @@
           <t>operator1@company.com</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>2</v>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>11.040756, 77.030313</t>
+        </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>PREV-1002</t>
+          <t>89/1, Avinashi Road, Saravanampatty, Coimbatore</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>11.040756, 77.030313</t>
+          <t>Avinashi Road</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>89/1, Avinashi Road, Saravanampatty, Coimbatore</t>
+          <t>Saravanampatty</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avinashi Road</t>
+          <t>Coimbatore North</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Saravanampatty</t>
+          <t>Coimbatore</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Coimbatore North</t>
+          <t>89/1</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Coimbatore</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>89/1</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Suresh Reddy</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
+          <t>2024-03-16</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
           <t>Commercial</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Vacant Plot</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>Suresh Reddy</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>2024-03-16</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Vacant Plot</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>Suresh Reddy</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
           <t>9876543211</t>
         </is>
       </c>
-      <c r="V3" s="2" t="inlineStr"/>
-      <c r="W3" s="2" t="inlineStr"/>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr">
         <is>
           <t>Vacant plot, no active construction observed</t>
         </is>

</xml_diff>